<commit_message>
Add record: フリー 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -7,10 +7,10 @@
   </bookViews>
   <sheets>
     <sheet name="メドレー" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="フリー" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ブレ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="バッタ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="バック" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ブレ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="バッタ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="バック" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -680,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50.61</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>49.82</v>
+        <v>66.84</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -781,11 +781,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>48.98</v>
+        <v>60.52</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45955</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -807,11 +807,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>46.9</v>
+        <v>56.15</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46033</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -833,11 +833,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44.07</v>
+        <v>57.26</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46075</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -859,11 +859,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>56.39</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -873,11 +873,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46130</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -889,21 +889,21 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>54.31</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46033</v>
+        <v>46180</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -911,11 +911,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42.36</v>
+        <v>53.01</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -925,11 +925,11 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46055</v>
+        <v>46187</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>41.5</v>
+        <v>52.53</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -951,11 +951,11 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>46075</v>
+        <v>46207</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -967,139 +967,9 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>42.24</v>
+        <v>53.65</v>
       </c>
       <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>40.06</v>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1116,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1153,7 +1023,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45823</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1169,7 +1039,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>68.26000000000001</v>
+        <v>58.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1179,7 +1049,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45956</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1191,11 +1061,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>66.84</v>
+        <v>52.07</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1205,7 +1075,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45844</v>
+        <v>45984</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1221,7 +1091,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>60.52</v>
+        <v>51.12</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1231,7 +1101,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45955</v>
+        <v>46033</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1247,7 +1117,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>56.15</v>
+        <v>53</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1257,7 +1127,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46033</v>
+        <v>46055</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1273,7 +1143,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>57.26</v>
+        <v>49.85</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1299,7 +1169,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>56.39</v>
+        <v>53.89</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1321,11 +1191,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>54.31</v>
+        <v>52.64</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1335,7 +1205,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46180</v>
+        <v>46152</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1347,21 +1217,21 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>53.01</v>
+        <v>49.1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46187</v>
+        <v>46208</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1373,39 +1243,13 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>52.53</v>
+        <v>49.43</v>
       </c>
       <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>53.65</v>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1422,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1459,7 +1303,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1475,7 +1319,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.49</v>
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1485,7 +1329,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1497,11 +1341,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52.07</v>
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1511,7 +1355,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1523,11 +1367,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51.12</v>
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1537,7 +1381,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1549,11 +1393,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1563,7 +1407,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1575,11 +1419,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.85</v>
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1589,7 +1433,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1601,11 +1445,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>49.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1615,11 +1459,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46130</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1627,25 +1471,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52.64</v>
+        <v>50.03</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46152</v>
+        <v>46055</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1657,35 +1501,165 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>49.1</v>
+        <v>48.34</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>46.76</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
         <v>46208</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>49.43</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="C15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1702,7 +1676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1755,7 +1729,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.72</v>
+        <v>50.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1765,7 +1739,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1781,7 +1755,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>56.3</v>
+        <v>49.82</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1807,7 +1781,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>55.74</v>
+        <v>48.98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1833,7 +1807,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>56.07</v>
+        <v>46.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1859,7 +1833,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>52.11</v>
+        <v>44.07</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1869,7 +1843,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45956</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1885,7 +1859,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.12</v>
+        <v>43.01</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1911,7 +1885,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>50.03</v>
+        <v>42.75</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1921,7 +1895,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46055</v>
+        <v>46033</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1937,7 +1911,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>48.34</v>
+        <v>42.36</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1947,7 +1921,7 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46075</v>
+        <v>46055</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1959,11 +1933,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>48.9</v>
+        <v>41.5</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1973,11 +1947,11 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>46130</v>
+        <v>46075</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1985,21 +1959,21 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>48.72</v>
+        <v>42.24</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>46152</v>
+        <v>46130</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -2015,17 +1989,17 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>45.85</v>
+        <v>40.99</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>46179</v>
+        <v>46152</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2037,11 +2011,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>47.75</v>
+        <v>39.25</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -2051,7 +2025,7 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>46187</v>
+        <v>46180</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2063,11 +2037,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46.76</v>
+        <v>40.89</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2077,7 +2051,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>46208</v>
+        <v>46187</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2089,15 +2063,67 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>47.77</v>
+        <v>39.76</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add record: フリー 200m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -1676,7 +1676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,6 +2231,32 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add record: メドレー 200m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="メドレー" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ブレ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="バッタ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="バック" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="バッタ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="バック" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="メドレー" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,35 +505,33 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小3</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'52"00</t>
-        </is>
+      <c r="E2" t="n">
+        <v>68.26000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45808</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -541,27 +539,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'17"24</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>66.84</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45899</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -569,27 +565,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'50"98</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>60.52</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45991</v>
+        <v>45955</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -597,27 +591,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'44"22</t>
-        </is>
+      <c r="E5" t="n">
+        <v>56.15</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46081</v>
+        <v>46033</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -625,47 +617,149 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'35"70</t>
-        </is>
+      <c r="E6" t="n">
+        <v>57.26</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46172</v>
+        <v>46075</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>207.18</v>
+        <v>56.39</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>54.31</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>53.01</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>52.53</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>53.65</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -680,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,7 +811,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45823</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -733,7 +827,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>68.26000000000001</v>
+        <v>58.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -743,7 +837,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45956</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -755,11 +849,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>66.84</v>
+        <v>52.07</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -769,7 +863,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45844</v>
+        <v>45984</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -785,7 +879,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>60.52</v>
+        <v>51.12</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -795,7 +889,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45955</v>
+        <v>46033</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -811,7 +905,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>56.15</v>
+        <v>53</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -821,7 +915,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46033</v>
+        <v>46055</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -837,7 +931,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>57.26</v>
+        <v>49.85</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -863,7 +957,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>56.39</v>
+        <v>53.89</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -885,11 +979,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>54.31</v>
+        <v>52.64</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -899,7 +993,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46180</v>
+        <v>46152</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -911,21 +1005,21 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>53.01</v>
+        <v>49.1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46187</v>
+        <v>46208</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -937,39 +1031,13 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>52.53</v>
+        <v>49.43</v>
       </c>
       <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>53.65</v>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -986,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1023,7 +1091,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1039,7 +1107,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.49</v>
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1049,7 +1117,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1061,11 +1129,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52.07</v>
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1075,7 +1143,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1087,11 +1155,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51.12</v>
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1101,7 +1169,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1113,11 +1181,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1127,7 +1195,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1139,11 +1207,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.85</v>
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1153,7 +1221,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1165,11 +1233,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>49.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1179,11 +1247,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46130</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1191,25 +1259,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52.64</v>
+        <v>50.03</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46152</v>
+        <v>46055</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1221,35 +1289,165 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>49.1</v>
+        <v>48.34</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>46.76</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
         <v>46208</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>長水路</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>49.43</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E15" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1266,7 +1464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1319,7 +1517,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.72</v>
+        <v>50.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1329,7 +1527,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1345,7 +1543,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>56.3</v>
+        <v>49.82</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1371,7 +1569,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>55.74</v>
+        <v>48.98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1397,7 +1595,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>56.07</v>
+        <v>46.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1423,7 +1621,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>52.11</v>
+        <v>44.07</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1433,7 +1631,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45956</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1449,7 +1647,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.12</v>
+        <v>43.01</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1475,7 +1673,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>50.03</v>
+        <v>42.75</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1485,7 +1683,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46055</v>
+        <v>46033</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1501,7 +1699,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>48.34</v>
+        <v>42.36</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1511,7 +1709,7 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46075</v>
+        <v>46055</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1523,11 +1721,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>48.9</v>
+        <v>41.5</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1537,11 +1735,11 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>46130</v>
+        <v>46075</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1549,21 +1747,21 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>48.72</v>
+        <v>42.24</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>46152</v>
+        <v>46130</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1579,17 +1777,17 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>45.85</v>
+        <v>40.99</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>46179</v>
+        <v>46152</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1601,11 +1799,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>47.75</v>
+        <v>39.25</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1615,7 +1813,7 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>46187</v>
+        <v>46180</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1627,11 +1825,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46.76</v>
+        <v>40.89</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1641,7 +1839,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>46208</v>
+        <v>46187</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1653,15 +1851,197 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>長水路</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>47.77</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
+      <c r="E16" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>50</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>50</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
@@ -1676,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1713,33 +2093,35 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>50.61</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'52"00</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1747,25 +2129,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>49.82</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'17"24</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1773,25 +2157,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>48.98</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'50"98</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1799,25 +2185,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>46.9</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'44"22</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1825,33 +2213,35 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>44.07</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'35"70</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46172</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1859,399 +2249,35 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>207.18</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>205.74</v>
       </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>42.36</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>42.24</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>40.06</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>50</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>50</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>50</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>50</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>200</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F22" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>

</xml_diff>

<commit_message>
Delete record: フリー 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -9,8 +9,8 @@
     <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="バッタ" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="バック" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="メドレー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="メドレー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1464,7 +1464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1501,33 +1501,35 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>50.61</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'52"00</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1535,25 +1537,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>49.82</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'17"24</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1561,25 +1565,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>48.98</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'50"98</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1587,25 +1593,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>46.9</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'44"22</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1613,33 +1621,35 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>44.07</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'35"70</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46172</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1647,399 +1657,35 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>207.18</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>205.74</v>
       </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>42.36</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>42.24</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>40.06</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>50</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>50</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>50</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>50</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>200</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F22" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
@@ -2056,7 +1702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2093,35 +1739,33 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小3</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'52"00</t>
-        </is>
+      <c r="E2" t="n">
+        <v>50.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45808</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -2129,27 +1773,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'17"24</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>49.82</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45899</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2157,27 +1799,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'50"98</t>
-        </is>
+      <c r="E4" t="n">
+        <v>48.98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45991</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -2185,27 +1825,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'44"22</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>46.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46081</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -2213,35 +1851,33 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'35"70</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>44.07</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46172</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2249,35 +1885,373 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>207.18</v>
+        <v>43.01</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>42.24</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>40.99</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>40.89</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
         <v>46264</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>50</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>205.74</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>200</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
         <v>205.74</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>

</xml_diff>

<commit_message>
Delete record: フリー 200m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -1702,7 +1702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2127,32 +2127,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>200</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add record: バッタ 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -7,10 +7,10 @@
   </bookViews>
   <sheets>
     <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="バッタ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="バック" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="メドレー" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="バック" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="バッタ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -774,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,7 +811,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.49</v>
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -849,11 +849,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52.07</v>
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -875,11 +875,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51.12</v>
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -901,11 +901,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -927,11 +927,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.85</v>
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -953,11 +953,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>49.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -967,11 +967,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46130</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -979,25 +979,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52.64</v>
+        <v>50.03</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46152</v>
+        <v>46055</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1009,35 +1009,165 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>49.1</v>
+        <v>48.34</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>46.76</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
         <v>46208</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>49.43</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="C15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1054,7 +1184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1091,33 +1221,35 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>58.72</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'52"00</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1125,25 +1257,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>56.3</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'17"24</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1151,25 +1285,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>55.74</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'50"98</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1177,25 +1313,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>56.07</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'44"22</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1203,33 +1341,35 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>52.11</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'35"70</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45956</v>
+        <v>46172</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1237,219 +1377,37 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.12</v>
+        <v>207.18</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>50.03</v>
+        <v>205.74</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>48.34</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>48.72</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
           <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>45.85</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>46.76</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>46208</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>47.77</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1501,35 +1459,33 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小3</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'52"00</t>
-        </is>
+      <c r="E2" t="n">
+        <v>50.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45808</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1537,27 +1493,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'17"24</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>49.82</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45899</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1565,27 +1519,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'50"98</t>
-        </is>
+      <c r="E4" t="n">
+        <v>48.98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45991</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1593,27 +1545,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'44"22</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>46.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46081</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1621,35 +1571,33 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'35"70</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>44.07</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46172</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1657,37 +1605,245 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>207.18</v>
+        <v>43.01</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46264</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>42.24</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>205.74</v>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>40.99</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>40.89</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1739,7 +1895,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45823</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1755,7 +1911,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50.61</v>
+        <v>58.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1765,7 +1921,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45956</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1777,11 +1933,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>49.82</v>
+        <v>52.07</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1791,7 +1947,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45984</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1803,11 +1959,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>48.98</v>
+        <v>51.12</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1817,7 +1973,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>46033</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1829,11 +1985,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>46.9</v>
+        <v>53</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1843,7 +1999,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46055</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1855,11 +2011,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44.07</v>
+        <v>49.85</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1869,7 +2025,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46075</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1881,11 +2037,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>53.89</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1895,11 +2051,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46130</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1907,25 +2063,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>52.64</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46033</v>
+        <v>46152</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1937,21 +2093,21 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42.36</v>
+        <v>49.1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46055</v>
+        <v>46208</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1959,11 +2115,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>41.5</v>
+        <v>49.43</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1973,11 +2129,11 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>46075</v>
+        <v>46313</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1989,139 +2145,9 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>42.24</v>
+        <v>48.25</v>
       </c>
       <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>39.76</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>46207</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>40.06</v>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>

</xml_diff>